<commit_message>
Added Beyond This MVP section, embedded delivery-plan previews, added US-11 concept item
</commit_message>
<xml_diff>
--- a/data/Project_Delivery_Plan.xlsx
+++ b/data/Project_Delivery_Plan.xlsx
@@ -13,6 +13,8 @@
     <sheet name="Risk_Dependency_Tracker" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Change_Management_Plan" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Sprint_Backlog" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Functional_Spec_US-02" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="AI_Assisted_UAT_Notes" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="302">
   <si>
     <t xml:space="preserve">User Stories: Equipment / Tool Request Approval</t>
   </si>
@@ -587,6 +589,21 @@
     <t xml:space="preserve">- One change champion per department: not the BA, a peer who models the new process and answers informal questions.</t>
   </si>
   <si>
+    <t xml:space="preserve">Multi-Site Rollout Considerations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Micron operates fabs and sites across multiple US locations (Boise ID, Manassas VA, Syracuse NY expansion) and internationally (Hiroshima Japan, Taiwan, Singapore, Sanand India). A single-timezone, single-champion rollout plan does not scale to that footprint. Adjustments for actual rollout:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Change champion assigned per site, not per department alone; a Boise-based champion cannot cover a Syracuse shift's informal questions in real time.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Office hours (Phase 1) held at times that cover at least two major timezones, or recorded and made async-available for fab shift workers who are not at a desk during standard office hours.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Wave sequencing (Phase 3) treats each site as its own wave, not a single global cutover, since local ServiceNow configuration and cost-center mappings differ by site.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Adoption Metrics (defined before rollout, not after)</t>
   </si>
   <si>
@@ -695,7 +712,226 @@
     <t xml:space="preserve">Backlog</t>
   </si>
   <si>
+    <t xml:space="preserve">Backlog (concept only, not scoped)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US-11 (stretch)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Predictive request initiation: system flags likely equipment needs from usage/lifecycle data and drafts a request for the employee to confirm, instead of waiting for a manual submission. This would be genuinely agentic (autonomous, adaptive), not rule-based like US-01 through US-09. Not scoped, not pointed, not part of this MVP. See README, 'Beyond This MVP.'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concept</t>
+  </si>
+  <si>
     <t xml:space="preserve">Scheduled points: 36 (US-01 through US-09, excluding backlog item US-10).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional Specification: Policy &amp; Budget Validation (US-02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The one story in the backlog with real business-rule complexity. User stories say what the system should do; this says exactly how.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Overview</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When an employee submits an equipment/tool request via the self-service portal, the system must automatically validate it against two rule sets, budget availability and catalog/policy compliance, before routing to an approver. This replaces the manual policy check currently performed informally by the approving manager.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Trigger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Request submission event (US-01 complete) fires the validation service.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Inputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Requested item (catalog SKU or free-text description)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Requested cost (catalog price or manual estimate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Requester's cost center and employee ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Fiscal year / quarter (for budget period lookup)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Business Rules</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Result</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BR-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item matches approved catalog SKU AND cost &lt;= department's remaining quarterly budget</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto-proceed to routing (US-03), no manual review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BR-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost exceeds department's remaining quarterly budget</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status = Budget Review Required; routes to requester's manager AND Finance Systems Liaison</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BR-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item does not match an approved catalog SKU (non-standard request)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status = Policy Review Required; routes to manager with policy-exception note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BR-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Both BR-2 and BR-3 conditions true</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status = Combined Review Required; routes to manager, Finance Systems Liaison, and a Digital Workplace analyst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BR-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Budget remaining calculation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approved quarterly budget minus sum of already-approved requests this quarter, including pending Budget Review Required requests not yet rejected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Outputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Request status field updated (Auto-Approved-Pending-Routing / Budget-Review-Required / Policy-Review-Required / Combined-Review-Required)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Audit log entry: rule(s) triggered, timestamp, evaluated budget figures</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Notification to requester confirming validation outcome (not full approval)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Exception Handling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Budget data unavailable (new cost center, sync failure): request held in Data Pending status, routed to Finance Systems Liaison with a 24-hour SLA (ties to R-02 in the risk tracker).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Catalog data stale (item recently deprecated): flagged for manual catalog review, not silently blocked.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. Data Dependencies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Real-time or near-real-time department budget balance feed (owned by Finance Systems)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Current approved-catalog list (owned by Procurement / IT Asset Management)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Cost-center hierarchy mapping (owned by HR / Finance)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8. Non-Functional Requirements</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Validation completes within 60 seconds of submission (supports the under-1-minute routing target in US-03's acceptance criteria).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- All rule evaluations logged for audit purposes; real spend is involved, which makes this a financial control, not just a workflow step.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9. Open Questions (flagged, not resolved)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Is remaining budget checked at cost-center level or program level? Assumed cost-center level here; needs confirmation with the Finance Systems Liaison before build (ties to R-02).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Does a rejected Budget Review Required request release its reserved budget immediately, or is there a hold period? Not yet defined.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Where AI Actually Helped (and Where It Didn't)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Writing test cases from user stories is repetitive, first-draft work. That's a real fit for an LLM. This shows the exact prompt used, what came back, and what a human still had to catch.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prompt used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Given this user story and its acceptance criteria, draft 2-3 UAT test cases. Format: Test ID, Scenario, Steps, Expected Result. Story: US-09, As an approver, I want to reject a request with a stated reason so that the requester understands why it did not proceed, instead of the request simply stalling. Acceptance criteria: Given a routed request, when the approver selects Reject and enters a reason, then the requester is notified with that reason and the ticket closes as Rejected, not left open or auto-escalated."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raw AI-drafted output (unedited)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reject a request</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approver opens the request and selects Reject.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The request is rejected.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reject without a reason</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approver selects Reject and leaves the reason field blank.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">System prompts the approver to enter a reason before proceeding.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What a human had to catch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missed the actual point of the story</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-A's "the request is rejected" is generic. It never tests the one behavior US-09 exists to guarantee: that a rejected ticket does not auto-escalate, which was the real gap (R-07) found during test planning. A generic AI-drafted test case can pass while missing the requirement it was supposed to verify.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invented behavior not in the spec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-B assumes the system enforces a mandatory reason field with a blocking prompt. Nothing in the acceptance criteria says that. Keeping this test case would have shipped a requirement nobody actually wrote. It was dropped rather than kept "just in case."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What shipped instead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-12 in UAT_Test_Plan explicitly tests: "Requester notified with the reason; ticket closes as Rejected, does not escalate." That distinguishing detail came from re-reading the acceptance criteria against what R-07 was actually flagging, not from the AI draft.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Where this generalizes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LLM-drafted first passes are a real time-saver for volume, boilerplate test structure, and covering the obvious happy path. They are not a substitute for knowing which single test case actually matters for a given story, or for noticing when a draft has quietly invented a requirement. On this team, the useful pattern is: AI drafts, a person checks the draft against the actual risk it's supposed to catch, not just against the story text.</t>
   </si>
 </sst>
 </file>
@@ -705,7 +941,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -769,6 +1005,21 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FFB23A48"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -837,7 +1088,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -874,7 +1125,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -906,7 +1177,7 @@
       <rgbColor rgb="FFCCCCCC"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFB23A48"/>
       <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
@@ -2032,7 +2303,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="60"/>
@@ -2183,32 +2454,77 @@
         <v>187</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="s">
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+    </row>
+    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9" t="s">
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+    </row>
+    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="s">
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+    </row>
+    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
         <v>191</v>
       </c>
+      <c r="B21" s="8"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="7" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="10" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="10" t="s">
+        <v>196</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="8">
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A21:E21"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2225,7 +2541,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
@@ -2237,26 +2553,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>121</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>60</v>
@@ -2264,245 +2580,262 @@
     </row>
     <row r="5" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>8</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>5</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>8</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>17</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>5</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>206</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="D10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>25</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="D11" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>30</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="D12" s="4" t="n">
         <v>5</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="D13" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>34</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="D14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>38</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>46</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="D18" s="4" t="n">
         <v>8</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
-        <v>223</v>
+        <v>227</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -2514,4 +2847,517 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E44"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+    </row>
+    <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11" t="s">
+        <v>241</v>
+      </c>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+    </row>
+    <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11" t="s">
+        <v>242</v>
+      </c>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+    </row>
+    <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="E18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="E19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="12" t="s">
+        <v>254</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="E20" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="E21" s="5"/>
+    </row>
+    <row r="22" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="E22" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="7" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
+    </row>
+    <row r="26" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="B26" s="11"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
+    </row>
+    <row r="27" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="11"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="11" t="s">
+        <v>268</v>
+      </c>
+      <c r="B30" s="11"/>
+      <c r="C30" s="11"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="11"/>
+    </row>
+    <row r="31" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="11" t="s">
+        <v>269</v>
+      </c>
+      <c r="B31" s="11"/>
+      <c r="C31" s="11"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="11"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="7" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="11" t="s">
+        <v>271</v>
+      </c>
+      <c r="B34" s="11"/>
+      <c r="C34" s="11"/>
+      <c r="D34" s="11"/>
+      <c r="E34" s="11"/>
+    </row>
+    <row r="35" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="11" t="s">
+        <v>272</v>
+      </c>
+      <c r="B35" s="11"/>
+      <c r="C35" s="11"/>
+      <c r="D35" s="11"/>
+      <c r="E35" s="11"/>
+    </row>
+    <row r="36" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="11" t="s">
+        <v>273</v>
+      </c>
+      <c r="B36" s="11"/>
+      <c r="C36" s="11"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="7" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="B39" s="11"/>
+      <c r="C39" s="11"/>
+      <c r="D39" s="11"/>
+      <c r="E39" s="11"/>
+    </row>
+    <row r="40" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="B40" s="11"/>
+      <c r="C40" s="11"/>
+      <c r="D40" s="11"/>
+      <c r="E40" s="11"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="7" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="11" t="s">
+        <v>278</v>
+      </c>
+      <c r="B43" s="11"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="11"/>
+      <c r="E43" s="11"/>
+    </row>
+    <row r="44" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="B44" s="11"/>
+      <c r="C44" s="11"/>
+      <c r="D44" s="11"/>
+      <c r="E44" s="11"/>
+    </row>
+  </sheetData>
+  <mergeCells count="28">
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A40:E40"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A44:E44"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E23"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="13" t="s">
+        <v>283</v>
+      </c>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="14" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="11" t="s">
+        <v>295</v>
+      </c>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="14" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11" t="s">
+        <v>297</v>
+      </c>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="11" t="s">
+        <v>299</v>
+      </c>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11" t="s">
+        <v>301</v>
+      </c>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A23:E23"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>